<commit_message>
feat: final production hierarchy - designation-based names from Rank Master
</commit_message>
<xml_diff>
--- a/management_hierarchy.xlsx
+++ b/management_hierarchy.xlsx
@@ -397,13 +397,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
     <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" customWidth="1"/>
     <col min="8" max="8" width="15.83203125" customWidth="1"/>
@@ -420,7 +420,7 @@
         <v>Agent Code</v>
       </c>
       <c r="D1" t="str">
-        <v>Sponsor Agent Code</v>
+        <v>Sponsor</v>
       </c>
       <c r="E1" t="str">
         <v>Login Email</v>
@@ -437,215 +437,241 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Rajesh Kumar</v>
+        <v>Super Admin</v>
       </c>
       <c r="B2">
-        <v>18</v>
+        <v>99</v>
       </c>
       <c r="C2" t="str">
-        <v>MGT000018</v>
+        <v>SUPER-ADMIN</v>
       </c>
       <c r="D2" t="str">
+        <v>Root</v>
+      </c>
+      <c r="E2" t="str">
         <v>admin@apex.com</v>
       </c>
-      <c r="E2" t="str">
-        <v>rajesh.kumar@apex.local</v>
-      </c>
       <c r="F2" t="str">
-        <v>Rajesh@Apex2026</v>
+        <v>Apex@12345</v>
       </c>
       <c r="G2" t="str">
-        <v>9876543210</v>
+        <v>N/A</v>
       </c>
       <c r="H2" t="str">
-        <v>ABCDE1234F</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Sanjay Singhal</v>
+        <v>Managing Director</v>
       </c>
       <c r="B3">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" t="str">
-        <v>MGT000017</v>
+        <v>MGT000018</v>
       </c>
       <c r="D3" t="str">
-        <v>MGT000018</v>
+        <v>admin@apex.com</v>
       </c>
       <c r="E3" t="str">
-        <v>sanjay.singhal@apex.local</v>
+        <v>mgd@apex.local</v>
       </c>
       <c r="F3" t="str">
-        <v>Sanjay@Apex2026</v>
+        <v>MGD@Apex2026</v>
       </c>
       <c r="G3" t="str">
-        <v>9876543211</v>
+        <v>9800000018</v>
       </c>
       <c r="H3" t="str">
-        <v>BCDEF2345G</v>
+        <v>MGDIR0018A</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Vikram Malhotra</v>
+        <v>Executive Vice President</v>
       </c>
       <c r="B4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" t="str">
-        <v>MGT000016</v>
+        <v>MGT000017</v>
       </c>
       <c r="D4" t="str">
-        <v>MGT000017</v>
+        <v>MGT000018</v>
       </c>
       <c r="E4" t="str">
-        <v>vikram.malhotra@apex.local</v>
+        <v>evp@apex.local</v>
       </c>
       <c r="F4" t="str">
-        <v>Vikram@Apex2026</v>
+        <v>EVP@Apex2026</v>
       </c>
       <c r="G4" t="str">
-        <v>9876543212</v>
+        <v>9800000017</v>
       </c>
       <c r="H4" t="str">
-        <v>CDEFG3456H</v>
+        <v>EVPRE0017B</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Sunita Deshmukh</v>
+        <v>Senior Vice President</v>
       </c>
       <c r="B5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" t="str">
-        <v>MGT000015</v>
+        <v>MGT000016</v>
       </c>
       <c r="D5" t="str">
-        <v>MGT000016</v>
+        <v>MGT000017</v>
       </c>
       <c r="E5" t="str">
-        <v>sunita.deshmukh@apex.local</v>
+        <v>svp@apex.local</v>
       </c>
       <c r="F5" t="str">
-        <v>Sunita@Apex2026</v>
+        <v>SVP@Apex2026</v>
       </c>
       <c r="G5" t="str">
-        <v>9876543213</v>
+        <v>9800000016</v>
       </c>
       <c r="H5" t="str">
-        <v>DEFGH4567I</v>
+        <v>SVPRE0016C</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Pankaj Mishra</v>
+        <v>Vice President</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" t="str">
-        <v>MGT000014</v>
+        <v>MGT000015</v>
       </c>
       <c r="D6" t="str">
-        <v>MGT000015</v>
+        <v>MGT000016</v>
       </c>
       <c r="E6" t="str">
-        <v>pankaj.mishra@apex.local</v>
+        <v>vp@apex.local</v>
       </c>
       <c r="F6" t="str">
-        <v>Pankaj@Apex2026</v>
+        <v>VP@Apex20261</v>
       </c>
       <c r="G6" t="str">
-        <v>9876543214</v>
+        <v>9800000015</v>
       </c>
       <c r="H6" t="str">
-        <v>EFGHI5678J</v>
+        <v>VPPRE0015D</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Aarav Mehta</v>
+        <v>Asst. Vice President</v>
       </c>
       <c r="B7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7" t="str">
-        <v>MGT000013</v>
+        <v>MGT000014</v>
       </c>
       <c r="D7" t="str">
-        <v>MGT000014</v>
+        <v>MGT000015</v>
       </c>
       <c r="E7" t="str">
-        <v>aarav.mehta@apex.local</v>
+        <v>avp@apex.local</v>
       </c>
       <c r="F7" t="str">
-        <v>Aarav@Apex2026</v>
+        <v>AVP@Apex2026</v>
       </c>
       <c r="G7" t="str">
-        <v>9876543215</v>
+        <v>9800000014</v>
       </c>
       <c r="H7" t="str">
-        <v>FGHIJ6789K</v>
+        <v>AVPRE0014E</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Deepak Joshi</v>
+        <v>Chief Marketing Director</v>
       </c>
       <c r="B8">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" t="str">
-        <v>MGT000012</v>
+        <v>MGT000013</v>
       </c>
       <c r="D8" t="str">
-        <v>MGT000013</v>
+        <v>MGT000014</v>
       </c>
       <c r="E8" t="str">
-        <v>deepak.joshi@apex.local</v>
+        <v>cmd@apex.local</v>
       </c>
       <c r="F8" t="str">
-        <v>Deepak@Apex2026</v>
+        <v>CMD@Apex2026</v>
       </c>
       <c r="G8" t="str">
-        <v>9876543216</v>
+        <v>9800000013</v>
       </c>
       <c r="H8" t="str">
-        <v>GHIJK7890L</v>
+        <v>CMDRE0013F</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Neha Sharma</v>
+        <v>Marketing Director</v>
       </c>
       <c r="B9">
+        <v>12</v>
+      </c>
+      <c r="C9" t="str">
+        <v>MGT000012</v>
+      </c>
+      <c r="D9" t="str">
+        <v>MGT000013</v>
+      </c>
+      <c r="E9" t="str">
+        <v>md@apex.local</v>
+      </c>
+      <c r="F9" t="str">
+        <v>MD@Apex20261</v>
+      </c>
+      <c r="G9" t="str">
+        <v>9800000012</v>
+      </c>
+      <c r="H9" t="str">
+        <v>MDPRE0012G</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Sr. Executive Director</v>
+      </c>
+      <c r="B10">
         <v>11</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C10" t="str">
         <v>MGT000011</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D10" t="str">
         <v>MGT000012</v>
       </c>
-      <c r="E9" t="str">
-        <v>neha.sharma@apex.local</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Neha@Apex2026</v>
-      </c>
-      <c r="G9" t="str">
-        <v>9876543217</v>
-      </c>
-      <c r="H9" t="str">
-        <v>HIJKL8901M</v>
+      <c r="E10" t="str">
+        <v>sed@apex.local</v>
+      </c>
+      <c r="F10" t="str">
+        <v>SED@Apex2026</v>
+      </c>
+      <c r="G10" t="str">
+        <v>9800000011</v>
+      </c>
+      <c r="H10" t="str">
+        <v>SEDRE0011H</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>